<commit_message>
REF-LC: reserve-margin fix and NO_GAS_FLOOR (inputs of 22 Oct corrected run)
- custom_constraints.py: deduct retired coal from the reserve margin
  unconditionally. `coal_decom != 0` on a linopy expression returned a
  truthy Constraint, so retired coal was never removed (# MG adjusted).
- operational_constraints.xlsx: new NO_GAS_FLOOR label (NO_MIN_GAS without
  the 40%/30% monthly min-CF on new gas, H2-ready OCGT and ccgt_steam).
  NO_MIN_GAS unchanged.
- scenarios_to_run.xlsx: REF-LC regions 10 -> 1, operational_limits
  NO_MIN_GAS -> NO_GAS_FLOOR.

Known defect included (binary file, cannot be split): POL-6GW
transmission_grid 'existing+tdp' -> 'LC-2190h' (misplaced value,
validation checklist item 4). To be fixed with the POL rows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scenarios/Coal_Flexibilisation/scenarios_to_run.xlsx
+++ b/scenarios/Coal_Flexibilisation/scenarios_to_run.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1088" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1088" uniqueCount="207">
   <si>
     <t>index</t>
   </si>
@@ -199,37 +199,43 @@
     <t>DIESEL_LNG</t>
   </si>
   <si>
+    <t>NO_GAS_FLOOR</t>
+  </si>
+  <si>
+    <t>EAF_60</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>CT_2050</t>
+  </si>
+  <si>
+    <t>LOWDelEVs</t>
+  </si>
+  <si>
+    <t>RES_MRGN_10</t>
+  </si>
+  <si>
+    <t>BASE2</t>
+  </si>
+  <si>
+    <t>POL-2GW</t>
+  </si>
+  <si>
+    <t>2025, 2030, 2035, 2040, 2045, 2051</t>
+  </si>
+  <si>
     <t>NO_MIN_GAS</t>
   </si>
   <si>
-    <t>EAF_60</t>
-  </si>
-  <si>
-    <t>none</t>
-  </si>
-  <si>
-    <t>CT_2050</t>
-  </si>
-  <si>
-    <t>LOWDelEVs</t>
-  </si>
-  <si>
-    <t>RES_MRGN_10</t>
-  </si>
-  <si>
-    <t>BASE2</t>
-  </si>
-  <si>
-    <t>POL-2GW</t>
-  </si>
-  <si>
-    <t>2025, 2030, 2035, 2040, 2045, 2051</t>
-  </si>
-  <si>
     <t>POL-6GW</t>
   </si>
   <si>
     <t>2025, 2030, 2035, 2040, 2045, 2052</t>
+  </si>
+  <si>
+    <t>LC-2190h</t>
   </si>
   <si>
     <t>POL-16GW</t>
@@ -1302,7 +1308,7 @@
         <v>52</v>
       </c>
       <c r="L2" s="7">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="M2" s="8" t="s">
         <v>53</v>
@@ -1509,7 +1515,7 @@
         <v>61</v>
       </c>
       <c r="AK3" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL3" s="8" t="s">
         <v>59</v>
@@ -1544,7 +1550,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>48</v>
@@ -1557,7 +1563,7 @@
         <v>1</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J4" s="8" t="s">
         <v>51</v>
@@ -1578,7 +1584,7 @@
         <v>55</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="Q4" s="8" t="s">
         <v>57</v>
@@ -1641,7 +1647,7 @@
         <v>61</v>
       </c>
       <c r="AK4" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL4" s="8" t="s">
         <v>59</v>
@@ -1676,7 +1682,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>48</v>
@@ -1689,7 +1695,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J5" s="8" t="s">
         <v>51</v>
@@ -1773,7 +1779,7 @@
         <v>61</v>
       </c>
       <c r="AK5" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL5" s="8" t="s">
         <v>59</v>
@@ -1808,7 +1814,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>48</v>
@@ -1821,7 +1827,7 @@
         <v>1</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="J6" s="8" t="s">
         <v>51</v>
@@ -1905,7 +1911,7 @@
         <v>61</v>
       </c>
       <c r="AK6" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL6" s="8" t="s">
         <v>59</v>
@@ -1940,7 +1946,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>48</v>
@@ -1953,7 +1959,7 @@
         <v>1</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="J7" s="8" t="s">
         <v>51</v>
@@ -2037,7 +2043,7 @@
         <v>61</v>
       </c>
       <c r="AK7" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL7" s="8" t="s">
         <v>59</v>
@@ -2072,7 +2078,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>48</v>
@@ -2085,7 +2091,7 @@
         <v>1</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="J8" s="8" t="s">
         <v>51</v>
@@ -2169,7 +2175,7 @@
         <v>61</v>
       </c>
       <c r="AK8" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL8" s="8" t="s">
         <v>59</v>
@@ -2204,7 +2210,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>48</v>
@@ -2217,7 +2223,7 @@
         <v>1</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J9" s="8" t="s">
         <v>51</v>
@@ -2301,7 +2307,7 @@
         <v>61</v>
       </c>
       <c r="AK9" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL9" s="8" t="s">
         <v>59</v>
@@ -2336,7 +2342,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C10" s="8" t="s">
         <v>48</v>
@@ -2349,7 +2355,7 @@
         <v>1</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="J10" s="8" t="s">
         <v>51</v>
@@ -2433,7 +2439,7 @@
         <v>61</v>
       </c>
       <c r="AK10" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL10" s="8" t="s">
         <v>59</v>
@@ -2468,7 +2474,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>48</v>
@@ -2481,7 +2487,7 @@
         <v>1</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="J11" s="8" t="s">
         <v>51</v>
@@ -2565,7 +2571,7 @@
         <v>61</v>
       </c>
       <c r="AK11" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL11" s="8" t="s">
         <v>59</v>
@@ -2600,7 +2606,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>48</v>
@@ -2613,7 +2619,7 @@
         <v>1</v>
       </c>
       <c r="I12" s="8" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="J12" s="8" t="s">
         <v>51</v>
@@ -2697,7 +2703,7 @@
         <v>61</v>
       </c>
       <c r="AK12" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL12" s="8" t="s">
         <v>59</v>
@@ -2732,7 +2738,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>48</v>
@@ -2745,7 +2751,7 @@
         <v>1</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="J13" s="8" t="s">
         <v>51</v>
@@ -2829,7 +2835,7 @@
         <v>61</v>
       </c>
       <c r="AK13" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL13" s="8" t="s">
         <v>59</v>
@@ -2864,7 +2870,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>48</v>
@@ -2877,7 +2883,7 @@
         <v>1</v>
       </c>
       <c r="I14" s="8" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="J14" s="8" t="s">
         <v>51</v>
@@ -2961,7 +2967,7 @@
         <v>61</v>
       </c>
       <c r="AK14" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL14" s="8" t="s">
         <v>59</v>
@@ -2996,7 +3002,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C15" s="8" t="s">
         <v>48</v>
@@ -3009,7 +3015,7 @@
         <v>1</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J15" s="8" t="s">
         <v>51</v>
@@ -3093,7 +3099,7 @@
         <v>61</v>
       </c>
       <c r="AK15" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL15" s="8" t="s">
         <v>59</v>
@@ -3128,7 +3134,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C16" s="8" t="s">
         <v>48</v>
@@ -3141,7 +3147,7 @@
         <v>1</v>
       </c>
       <c r="I16" s="8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="J16" s="8" t="s">
         <v>51</v>
@@ -3225,7 +3231,7 @@
         <v>61</v>
       </c>
       <c r="AK16" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL16" s="8" t="s">
         <v>59</v>
@@ -3260,7 +3266,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C17" s="8" t="s">
         <v>48</v>
@@ -3273,7 +3279,7 @@
         <v>1</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="J17" s="8" t="s">
         <v>51</v>
@@ -3357,7 +3363,7 @@
         <v>61</v>
       </c>
       <c r="AK17" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL17" s="8" t="s">
         <v>59</v>
@@ -3392,7 +3398,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C18" s="8" t="s">
         <v>48</v>
@@ -3405,7 +3411,7 @@
         <v>1</v>
       </c>
       <c r="I18" s="8" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="J18" s="8" t="s">
         <v>51</v>
@@ -3489,7 +3495,7 @@
         <v>61</v>
       </c>
       <c r="AK18" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL18" s="8" t="s">
         <v>59</v>
@@ -3524,7 +3530,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C19" s="8" t="s">
         <v>48</v>
@@ -3537,7 +3543,7 @@
         <v>1</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="J19" s="8" t="s">
         <v>51</v>
@@ -3621,7 +3627,7 @@
         <v>61</v>
       </c>
       <c r="AK19" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL19" s="8" t="s">
         <v>59</v>
@@ -3656,7 +3662,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C20" s="8" t="s">
         <v>48</v>
@@ -3669,7 +3675,7 @@
         <v>1</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="J20" s="8" t="s">
         <v>51</v>
@@ -3753,7 +3759,7 @@
         <v>61</v>
       </c>
       <c r="AK20" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL20" s="8" t="s">
         <v>59</v>
@@ -3788,7 +3794,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C21" s="8" t="s">
         <v>48</v>
@@ -3801,7 +3807,7 @@
         <v>1</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="J21" s="8" t="s">
         <v>51</v>
@@ -3885,7 +3891,7 @@
         <v>61</v>
       </c>
       <c r="AK21" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL21" s="8" t="s">
         <v>59</v>
@@ -3919,276 +3925,276 @@
       <c r="A23" s="12"/>
       <c r="B23" s="13"/>
       <c r="C23" s="14" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E23" s="14" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="G23" s="14" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="H23" s="12" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="I23" s="14" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="J23" s="14" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="K23" s="14" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="L23" s="12" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="M23" s="14" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N23" s="14" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="O23" s="14" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P23" s="14" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="Q23" s="14" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="R23" s="14" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="S23" s="12" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="T23" s="12" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="U23" s="15" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="V23" s="15" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="W23" s="14" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="X23" s="14" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="Y23" s="14" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="Z23" s="14" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="AA23" s="14" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="AB23" s="14" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="AC23" s="15" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="AD23" s="14" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="AE23" s="14" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="AF23" s="14" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="AG23" s="14" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="AH23" s="14" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="AI23" s="14" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="AJ23" s="14" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="AK23" s="14" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="AL23" s="14" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="AM23" s="14" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="AN23" s="14" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="AO23" s="14" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="AP23" s="14" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="AQ23" s="14" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="AR23" s="14" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="AS23" s="14" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="AT23" s="14" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="24" ht="315" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A24" s="16"/>
       <c r="B24" s="17"/>
       <c r="C24" s="14" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F24" s="14" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G24" s="14" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H24" s="14" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="I24" s="14" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="J24" s="14" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K24" s="14" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="L24" s="14" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="M24" s="14" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="N24" s="14" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="O24" s="14" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="P24" s="14" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="Q24" s="14" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="R24" s="14" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="S24" s="14" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="T24" s="14" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="U24" s="14" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="V24" s="14" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="W24" s="14" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="X24" s="14" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="Y24" s="14" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="Z24" s="14" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="AA24" s="14" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="AB24" s="14" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="AC24" s="14" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="AD24" s="14" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="AE24" s="14" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="AF24" s="14" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="AG24" s="14" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="AH24" s="14" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="AI24" s="14" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="AJ24" s="14" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="AK24" s="14" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="AL24" s="14" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="AM24" s="14" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="AN24" s="14" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="AO24" s="14" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="AP24" s="14" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="AQ24" s="14"/>
       <c r="AR24" s="14" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="AS24" s="14" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="AT24" s="14" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="26" ht="18.75" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A26" s="7"/>
       <c r="B26" s="8" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C26" s="8" t="s">
         <v>48</v>
@@ -4203,13 +4209,13 @@
         <v>0</v>
       </c>
       <c r="G26" s="18" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="H26" s="7">
         <v>1</v>
       </c>
       <c r="I26" s="8" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="J26" s="8" t="s">
         <v>51</v>
@@ -4227,7 +4233,7 @@
         <v>54</v>
       </c>
       <c r="O26" s="9" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="P26" s="8" t="s">
         <v>56</v>
@@ -4293,7 +4299,7 @@
         <v>61</v>
       </c>
       <c r="AK26" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL26" s="8" t="s">
         <v>59</v>
@@ -4326,7 +4332,7 @@
     <row r="27" ht="18.75" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A27" s="7"/>
       <c r="B27" s="8" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C27" s="8" t="s">
         <v>48</v>
@@ -4347,7 +4353,7 @@
         <v>1</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="J27" s="8" t="s">
         <v>51</v>
@@ -4365,7 +4371,7 @@
         <v>54</v>
       </c>
       <c r="O27" s="9" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="P27" s="8" t="s">
         <v>56</v>
@@ -4431,7 +4437,7 @@
         <v>61</v>
       </c>
       <c r="AK27" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL27" s="8" t="s">
         <v>59</v>
@@ -4443,7 +4449,7 @@
         <v>63</v>
       </c>
       <c r="AO27" s="8" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="AP27" s="8" t="s">
         <v>64</v>
@@ -4464,7 +4470,7 @@
     <row r="28" ht="18.75" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A28" s="7"/>
       <c r="B28" s="8" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C28" s="8" t="s">
         <v>48</v>
@@ -4485,7 +4491,7 @@
         <v>1</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="J28" s="8" t="s">
         <v>51</v>
@@ -4503,7 +4509,7 @@
         <v>54</v>
       </c>
       <c r="O28" s="9" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="P28" s="8" t="s">
         <v>56</v>
@@ -4569,7 +4575,7 @@
         <v>61</v>
       </c>
       <c r="AK28" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL28" s="8" t="s">
         <v>59</v>
@@ -4584,7 +4590,7 @@
         <v>64</v>
       </c>
       <c r="AP28" s="8" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="AQ28" s="8" t="s">
         <v>64</v>
@@ -4602,7 +4608,7 @@
     <row r="29" ht="18.75" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A29" s="7"/>
       <c r="B29" s="8" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C29" s="8" t="s">
         <v>48</v>
@@ -4623,7 +4629,7 @@
         <v>1</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="J29" s="8" t="s">
         <v>51</v>
@@ -4641,7 +4647,7 @@
         <v>54</v>
       </c>
       <c r="O29" s="9" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="P29" s="8" t="s">
         <v>56</v>
@@ -4707,7 +4713,7 @@
         <v>61</v>
       </c>
       <c r="AK29" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL29" s="8" t="s">
         <v>59</v>
@@ -4719,10 +4725,10 @@
         <v>63</v>
       </c>
       <c r="AO29" s="8" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="AP29" s="8" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="AQ29" s="8" t="s">
         <v>64</v>
@@ -4740,7 +4746,7 @@
     <row r="30" ht="18.75" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A30" s="7"/>
       <c r="B30" s="8" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C30" s="8" t="s">
         <v>48</v>
@@ -4779,7 +4785,7 @@
         <v>54</v>
       </c>
       <c r="O30" s="9" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="P30" s="8" t="s">
         <v>56</v>
@@ -4845,7 +4851,7 @@
         <v>61</v>
       </c>
       <c r="AK30" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL30" s="8" t="s">
         <v>59</v>
@@ -4866,7 +4872,7 @@
         <v>64</v>
       </c>
       <c r="AR30" s="8" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="AS30" s="8" t="s">
         <v>67</v>
@@ -4878,7 +4884,7 @@
     <row r="31" ht="18.75" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A31" s="7"/>
       <c r="B31" s="8" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C31" s="8" t="s">
         <v>48</v>
@@ -4917,7 +4923,7 @@
         <v>54</v>
       </c>
       <c r="O31" s="9" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="P31" s="8" t="s">
         <v>56</v>
@@ -4983,7 +4989,7 @@
         <v>61</v>
       </c>
       <c r="AK31" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL31" s="8" t="s">
         <v>59</v>
@@ -4995,7 +5001,7 @@
         <v>63</v>
       </c>
       <c r="AO31" s="8" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="AP31" s="8" t="s">
         <v>64</v>
@@ -5004,7 +5010,7 @@
         <v>64</v>
       </c>
       <c r="AR31" s="8" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="AS31" s="8" t="s">
         <v>67</v>
@@ -5016,7 +5022,7 @@
     <row r="32" ht="18.75" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A32" s="7"/>
       <c r="B32" s="8" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C32" s="8" t="s">
         <v>48</v>
@@ -5055,7 +5061,7 @@
         <v>54</v>
       </c>
       <c r="O32" s="9" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="P32" s="8" t="s">
         <v>56</v>
@@ -5121,7 +5127,7 @@
         <v>61</v>
       </c>
       <c r="AK32" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL32" s="8" t="s">
         <v>59</v>
@@ -5142,7 +5148,7 @@
         <v>64</v>
       </c>
       <c r="AR32" s="8" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="AS32" s="8" t="s">
         <v>67</v>
@@ -5154,7 +5160,7 @@
     <row r="33" ht="18.75" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A33" s="7"/>
       <c r="B33" s="8" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C33" s="8" t="s">
         <v>48</v>
@@ -5193,7 +5199,7 @@
         <v>54</v>
       </c>
       <c r="O33" s="9" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="P33" s="8" t="s">
         <v>56</v>
@@ -5259,7 +5265,7 @@
         <v>61</v>
       </c>
       <c r="AK33" s="8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="AL33" s="8" t="s">
         <v>59</v>
@@ -5271,7 +5277,7 @@
         <v>63</v>
       </c>
       <c r="AO33" s="8" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="AP33" s="8" t="s">
         <v>65</v>
@@ -5280,7 +5286,7 @@
         <v>64</v>
       </c>
       <c r="AR33" s="8" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="AS33" s="8" t="s">
         <v>67</v>

</xml_diff>

<commit_message>
Complete four core gas-policy development scenarios and baseline validation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scenarios/Coal_Flexibilisation/scenarios_to_run.xlsx
+++ b/scenarios/Coal_Flexibilisation/scenarios_to_run.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1088" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1088" uniqueCount="206">
   <si>
     <t>index</t>
   </si>
@@ -233,9 +233,6 @@
   </si>
   <si>
     <t>2025, 2030, 2035, 2040, 2045, 2052</t>
-  </si>
-  <si>
-    <t>LC-2190h</t>
   </si>
   <si>
     <t>POL-16GW</t>
@@ -1105,7 +1102,7 @@
     <col min="15" max="15" width="15.142857142857142" customWidth="1"/>
     <col min="16" max="16" width="12.857142857142858" customWidth="1"/>
     <col min="17" max="17" width="14" customWidth="1"/>
-    <col min="18" max="18" width="20.857142857142858" customWidth="1"/>
+    <col min="18" max="18" width="28.285714285714285" customWidth="1"/>
     <col min="19" max="19" width="11" customWidth="1"/>
     <col min="20" max="20" width="25.285714285714285" customWidth="1"/>
     <col min="21" max="22" width="14" customWidth="1"/>
@@ -1131,6 +1128,7 @@
     <col min="44" max="44" width="15.571428571428571" customWidth="1"/>
     <col min="45" max="45" width="15.428571428571429" customWidth="1"/>
     <col min="46" max="46" width="15.857142857142858" customWidth="1"/>
+    <col min="47" max="92" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="32.25" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
@@ -1417,8 +1415,10 @@
       <c r="A3" s="7">
         <v>2</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>69</v>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>POL-3GW</t>
+        </is>
       </c>
       <c r="C3" s="8" t="s">
         <v>48</v>
@@ -1426,12 +1426,14 @@
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
       <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
+      <c r="G3" s="7">
+        <v>0</v>
+      </c>
       <c r="H3" s="7">
         <v>1</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="J3" s="8" t="s">
         <v>51</v>
@@ -1508,14 +1510,16 @@
       <c r="AH3" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="AI3" s="8" t="s">
-        <v>60</v>
+      <c r="AI3" s="8" t="inlineStr">
+        <is>
+          <t>3GW_GAS</t>
+        </is>
       </c>
       <c r="AJ3" s="8" t="s">
         <v>61</v>
       </c>
       <c r="AK3" s="8" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="AL3" s="8" t="s">
         <v>59</v>
@@ -1558,12 +1562,14 @@
       <c r="D4" s="7"/>
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
+      <c r="G4" s="7">
+        <v>0</v>
+      </c>
       <c r="H4" s="7">
         <v>1</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="J4" s="8" t="s">
         <v>51</v>
@@ -1584,7 +1590,7 @@
         <v>55</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="Q4" s="8" t="s">
         <v>57</v>
@@ -1640,14 +1646,16 @@
       <c r="AH4" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="AI4" s="8" t="s">
-        <v>60</v>
+      <c r="AI4" s="8" t="inlineStr">
+        <is>
+          <t>6GW_GAS</t>
+        </is>
       </c>
       <c r="AJ4" s="8" t="s">
         <v>61</v>
       </c>
       <c r="AK4" s="8" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="AL4" s="8" t="s">
         <v>59</v>
@@ -1681,8 +1689,10 @@
       <c r="A5" s="7">
         <v>4</v>
       </c>
-      <c r="B5" s="8" t="s">
-        <v>75</v>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>POL-18.25GW</t>
+        </is>
       </c>
       <c r="C5" s="8" t="s">
         <v>48</v>
@@ -1690,12 +1700,14 @@
       <c r="D5" s="7"/>
       <c r="E5" s="7"/>
       <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
+      <c r="G5" s="7">
+        <v>0</v>
+      </c>
       <c r="H5" s="7">
         <v>1</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>76</v>
+        <v>50</v>
       </c>
       <c r="J5" s="8" t="s">
         <v>51</v>
@@ -1772,14 +1784,16 @@
       <c r="AH5" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="AI5" s="8" t="s">
-        <v>60</v>
+      <c r="AI5" s="8" t="inlineStr">
+        <is>
+          <t>IRP25_GAS</t>
+        </is>
       </c>
       <c r="AJ5" s="8" t="s">
         <v>61</v>
       </c>
       <c r="AK5" s="8" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="AL5" s="8" t="s">
         <v>59</v>
@@ -1814,7 +1828,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>48</v>
@@ -1827,7 +1841,7 @@
         <v>1</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J6" s="8" t="s">
         <v>51</v>
@@ -1946,7 +1960,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>48</v>
@@ -1959,7 +1973,7 @@
         <v>1</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J7" s="8" t="s">
         <v>51</v>
@@ -2078,7 +2092,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>48</v>
@@ -2091,7 +2105,7 @@
         <v>1</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J8" s="8" t="s">
         <v>51</v>
@@ -2210,7 +2224,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>48</v>
@@ -2223,7 +2237,7 @@
         <v>1</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J9" s="8" t="s">
         <v>51</v>
@@ -2342,7 +2356,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C10" s="8" t="s">
         <v>48</v>
@@ -2355,7 +2369,7 @@
         <v>1</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J10" s="8" t="s">
         <v>51</v>
@@ -2474,7 +2488,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>48</v>
@@ -2487,7 +2501,7 @@
         <v>1</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J11" s="8" t="s">
         <v>51</v>
@@ -2606,7 +2620,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>48</v>
@@ -2619,7 +2633,7 @@
         <v>1</v>
       </c>
       <c r="I12" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J12" s="8" t="s">
         <v>51</v>
@@ -2738,7 +2752,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>48</v>
@@ -2751,7 +2765,7 @@
         <v>1</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J13" s="8" t="s">
         <v>51</v>
@@ -2870,7 +2884,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>48</v>
@@ -2883,7 +2897,7 @@
         <v>1</v>
       </c>
       <c r="I14" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="J14" s="8" t="s">
         <v>51</v>
@@ -3002,7 +3016,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C15" s="8" t="s">
         <v>48</v>
@@ -3015,7 +3029,7 @@
         <v>1</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J15" s="8" t="s">
         <v>51</v>
@@ -3134,7 +3148,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C16" s="8" t="s">
         <v>48</v>
@@ -3147,7 +3161,7 @@
         <v>1</v>
       </c>
       <c r="I16" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J16" s="8" t="s">
         <v>51</v>
@@ -3266,7 +3280,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C17" s="8" t="s">
         <v>48</v>
@@ -3279,7 +3293,7 @@
         <v>1</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J17" s="8" t="s">
         <v>51</v>
@@ -3398,7 +3412,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C18" s="8" t="s">
         <v>48</v>
@@ -3411,7 +3425,7 @@
         <v>1</v>
       </c>
       <c r="I18" s="8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J18" s="8" t="s">
         <v>51</v>
@@ -3530,7 +3544,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C19" s="8" t="s">
         <v>48</v>
@@ -3543,7 +3557,7 @@
         <v>1</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J19" s="8" t="s">
         <v>51</v>
@@ -3662,7 +3676,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C20" s="8" t="s">
         <v>48</v>
@@ -3675,7 +3689,7 @@
         <v>1</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="J20" s="8" t="s">
         <v>51</v>
@@ -3793,8 +3807,10 @@
       <c r="A21" s="7">
         <v>20</v>
       </c>
-      <c r="B21" s="8" t="s">
-        <v>72</v>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>POL-6GW_DUP</t>
+        </is>
       </c>
       <c r="C21" s="8" t="s">
         <v>48</v>
@@ -3802,12 +3818,14 @@
       <c r="D21" s="7"/>
       <c r="E21" s="7"/>
       <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
+      <c r="G21" s="7">
+        <v>0</v>
+      </c>
       <c r="H21" s="7">
         <v>1</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="J21" s="8" t="s">
         <v>51</v>
@@ -3925,276 +3943,276 @@
       <c r="A23" s="12"/>
       <c r="B23" s="13"/>
       <c r="C23" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="D23" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="D23" s="14" t="s">
+      <c r="E23" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="E23" s="14" t="s">
+      <c r="F23" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="F23" s="12" t="s">
+      <c r="G23" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="G23" s="14" t="s">
+      <c r="H23" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="H23" s="12" t="s">
+      <c r="I23" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="I23" s="14" t="s">
+      <c r="J23" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="J23" s="14" t="s">
+      <c r="K23" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="K23" s="14" t="s">
+      <c r="L23" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="L23" s="12" t="s">
+      <c r="M23" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="M23" s="14" t="s">
+      <c r="N23" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="N23" s="14" t="s">
+      <c r="O23" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="O23" s="14" t="s">
+      <c r="P23" s="14" t="s">
         <v>120</v>
       </c>
-      <c r="P23" s="14" t="s">
+      <c r="Q23" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="Q23" s="14" t="s">
+      <c r="R23" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="R23" s="14" t="s">
+      <c r="S23" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="S23" s="12" t="s">
+      <c r="T23" s="12" t="s">
         <v>124</v>
       </c>
-      <c r="T23" s="12" t="s">
+      <c r="U23" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="U23" s="15" t="s">
+      <c r="V23" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="V23" s="15" t="s">
+      <c r="W23" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="W23" s="14" t="s">
+      <c r="X23" s="14" t="s">
         <v>128</v>
       </c>
-      <c r="X23" s="14" t="s">
+      <c r="Y23" s="14" t="s">
         <v>129</v>
       </c>
-      <c r="Y23" s="14" t="s">
+      <c r="Z23" s="14" t="s">
         <v>130</v>
       </c>
-      <c r="Z23" s="14" t="s">
+      <c r="AA23" s="14" t="s">
         <v>131</v>
       </c>
-      <c r="AA23" s="14" t="s">
+      <c r="AB23" s="14" t="s">
         <v>132</v>
       </c>
-      <c r="AB23" s="14" t="s">
+      <c r="AC23" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="AC23" s="15" t="s">
+      <c r="AD23" s="14" t="s">
         <v>134</v>
       </c>
-      <c r="AD23" s="14" t="s">
+      <c r="AE23" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="AE23" s="14" t="s">
+      <c r="AF23" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="AF23" s="14" t="s">
+      <c r="AG23" s="14" t="s">
         <v>137</v>
       </c>
-      <c r="AG23" s="14" t="s">
+      <c r="AH23" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="AH23" s="14" t="s">
+      <c r="AI23" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="AI23" s="14" t="s">
+      <c r="AJ23" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="AJ23" s="14" t="s">
+      <c r="AK23" s="14" t="s">
         <v>141</v>
       </c>
-      <c r="AK23" s="14" t="s">
+      <c r="AL23" s="14" t="s">
         <v>142</v>
       </c>
-      <c r="AL23" s="14" t="s">
+      <c r="AM23" s="14" t="s">
         <v>143</v>
       </c>
-      <c r="AM23" s="14" t="s">
+      <c r="AN23" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="AN23" s="14" t="s">
+      <c r="AO23" s="14" t="s">
         <v>145</v>
       </c>
-      <c r="AO23" s="14" t="s">
+      <c r="AP23" s="14" t="s">
         <v>146</v>
       </c>
-      <c r="AP23" s="14" t="s">
+      <c r="AQ23" s="14" t="s">
         <v>147</v>
       </c>
-      <c r="AQ23" s="14" t="s">
+      <c r="AR23" s="14" t="s">
         <v>148</v>
       </c>
-      <c r="AR23" s="14" t="s">
+      <c r="AS23" s="14" t="s">
         <v>149</v>
       </c>
-      <c r="AS23" s="14" t="s">
+      <c r="AT23" s="14" t="s">
         <v>150</v>
-      </c>
-      <c r="AT23" s="14" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="24" ht="315" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A24" s="16"/>
       <c r="B24" s="17"/>
       <c r="C24" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="D24" s="14" t="s">
         <v>152</v>
       </c>
-      <c r="D24" s="14" t="s">
+      <c r="E24" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="F24" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="G24" s="14" t="s">
         <v>153</v>
       </c>
-      <c r="E24" s="14" t="s">
-        <v>153</v>
-      </c>
-      <c r="F24" s="14" t="s">
-        <v>153</v>
-      </c>
-      <c r="G24" s="14" t="s">
+      <c r="H24" s="14" t="s">
         <v>154</v>
       </c>
-      <c r="H24" s="14" t="s">
+      <c r="I24" s="14" t="s">
         <v>155</v>
       </c>
-      <c r="I24" s="14" t="s">
+      <c r="J24" s="14" t="s">
         <v>156</v>
       </c>
-      <c r="J24" s="14" t="s">
+      <c r="K24" s="14" t="s">
         <v>157</v>
       </c>
-      <c r="K24" s="14" t="s">
+      <c r="L24" s="14" t="s">
         <v>158</v>
       </c>
-      <c r="L24" s="14" t="s">
+      <c r="M24" s="14" t="s">
         <v>159</v>
       </c>
-      <c r="M24" s="14" t="s">
+      <c r="N24" s="14" t="s">
         <v>160</v>
       </c>
-      <c r="N24" s="14" t="s">
+      <c r="O24" s="14" t="s">
         <v>161</v>
       </c>
-      <c r="O24" s="14" t="s">
+      <c r="P24" s="14" t="s">
         <v>162</v>
       </c>
-      <c r="P24" s="14" t="s">
+      <c r="Q24" s="14" t="s">
         <v>163</v>
       </c>
-      <c r="Q24" s="14" t="s">
+      <c r="R24" s="14" t="s">
         <v>164</v>
       </c>
-      <c r="R24" s="14" t="s">
+      <c r="S24" s="14" t="s">
         <v>165</v>
       </c>
-      <c r="S24" s="14" t="s">
+      <c r="T24" s="14" t="s">
         <v>166</v>
       </c>
-      <c r="T24" s="14" t="s">
+      <c r="U24" s="14" t="s">
         <v>167</v>
       </c>
-      <c r="U24" s="14" t="s">
+      <c r="V24" s="14" t="s">
         <v>168</v>
       </c>
-      <c r="V24" s="14" t="s">
+      <c r="W24" s="14" t="s">
         <v>169</v>
       </c>
-      <c r="W24" s="14" t="s">
+      <c r="X24" s="14" t="s">
         <v>170</v>
       </c>
-      <c r="X24" s="14" t="s">
+      <c r="Y24" s="14" t="s">
         <v>171</v>
       </c>
-      <c r="Y24" s="14" t="s">
+      <c r="Z24" s="14" t="s">
         <v>172</v>
       </c>
-      <c r="Z24" s="14" t="s">
+      <c r="AA24" s="14" t="s">
         <v>173</v>
       </c>
-      <c r="AA24" s="14" t="s">
+      <c r="AB24" s="14" t="s">
         <v>174</v>
       </c>
-      <c r="AB24" s="14" t="s">
+      <c r="AC24" s="14" t="s">
         <v>175</v>
       </c>
-      <c r="AC24" s="14" t="s">
+      <c r="AD24" s="14" t="s">
         <v>176</v>
       </c>
-      <c r="AD24" s="14" t="s">
+      <c r="AE24" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="AE24" s="14" t="s">
+      <c r="AF24" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="AF24" s="14" t="s">
+      <c r="AG24" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="AG24" s="14" t="s">
+      <c r="AH24" s="14" t="s">
         <v>180</v>
       </c>
-      <c r="AH24" s="14" t="s">
+      <c r="AI24" s="14" t="s">
         <v>181</v>
       </c>
-      <c r="AI24" s="14" t="s">
+      <c r="AJ24" s="14" t="s">
         <v>182</v>
       </c>
-      <c r="AJ24" s="14" t="s">
+      <c r="AK24" s="14" t="s">
         <v>183</v>
       </c>
-      <c r="AK24" s="14" t="s">
+      <c r="AL24" s="14" t="s">
         <v>184</v>
       </c>
-      <c r="AL24" s="14" t="s">
+      <c r="AM24" s="14" t="s">
         <v>185</v>
       </c>
-      <c r="AM24" s="14" t="s">
+      <c r="AN24" s="14" t="s">
         <v>186</v>
       </c>
-      <c r="AN24" s="14" t="s">
+      <c r="AO24" s="14" t="s">
         <v>187</v>
       </c>
-      <c r="AO24" s="14" t="s">
+      <c r="AP24" s="14" t="s">
         <v>188</v>
-      </c>
-      <c r="AP24" s="14" t="s">
-        <v>189</v>
       </c>
       <c r="AQ24" s="14"/>
       <c r="AR24" s="14" t="s">
+        <v>189</v>
+      </c>
+      <c r="AS24" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="AS24" s="14" t="s">
+      <c r="AT24" s="14" t="s">
         <v>191</v>
-      </c>
-      <c r="AT24" s="14" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="26" ht="18.75" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A26" s="7"/>
       <c r="B26" s="8" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C26" s="8" t="s">
         <v>48</v>
@@ -4209,13 +4227,13 @@
         <v>0</v>
       </c>
       <c r="G26" s="18" t="s">
+        <v>193</v>
+      </c>
+      <c r="H26" s="7">
+        <v>1</v>
+      </c>
+      <c r="I26" s="8" t="s">
         <v>194</v>
-      </c>
-      <c r="H26" s="7">
-        <v>1</v>
-      </c>
-      <c r="I26" s="8" t="s">
-        <v>195</v>
       </c>
       <c r="J26" s="8" t="s">
         <v>51</v>
@@ -4233,7 +4251,7 @@
         <v>54</v>
       </c>
       <c r="O26" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="P26" s="8" t="s">
         <v>56</v>
@@ -4332,7 +4350,7 @@
     <row r="27" ht="18.75" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A27" s="7"/>
       <c r="B27" s="8" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C27" s="8" t="s">
         <v>48</v>
@@ -4353,7 +4371,7 @@
         <v>1</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="J27" s="8" t="s">
         <v>51</v>
@@ -4371,7 +4389,7 @@
         <v>54</v>
       </c>
       <c r="O27" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="P27" s="8" t="s">
         <v>56</v>
@@ -4449,7 +4467,7 @@
         <v>63</v>
       </c>
       <c r="AO27" s="8" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="AP27" s="8" t="s">
         <v>64</v>
@@ -4470,7 +4488,7 @@
     <row r="28" ht="18.75" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A28" s="7"/>
       <c r="B28" s="8" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C28" s="8" t="s">
         <v>48</v>
@@ -4491,7 +4509,7 @@
         <v>1</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="J28" s="8" t="s">
         <v>51</v>
@@ -4509,7 +4527,7 @@
         <v>54</v>
       </c>
       <c r="O28" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="P28" s="8" t="s">
         <v>56</v>
@@ -4590,7 +4608,7 @@
         <v>64</v>
       </c>
       <c r="AP28" s="8" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="AQ28" s="8" t="s">
         <v>64</v>
@@ -4608,7 +4626,7 @@
     <row r="29" ht="18.75" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A29" s="7"/>
       <c r="B29" s="8" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C29" s="8" t="s">
         <v>48</v>
@@ -4629,7 +4647,7 @@
         <v>1</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="J29" s="8" t="s">
         <v>51</v>
@@ -4647,7 +4665,7 @@
         <v>54</v>
       </c>
       <c r="O29" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="P29" s="8" t="s">
         <v>56</v>
@@ -4725,10 +4743,10 @@
         <v>63</v>
       </c>
       <c r="AO29" s="8" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="AP29" s="8" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="AQ29" s="8" t="s">
         <v>64</v>
@@ -4746,7 +4764,7 @@
     <row r="30" ht="18.75" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A30" s="7"/>
       <c r="B30" s="8" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C30" s="8" t="s">
         <v>48</v>
@@ -4785,7 +4803,7 @@
         <v>54</v>
       </c>
       <c r="O30" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="P30" s="8" t="s">
         <v>56</v>
@@ -4872,7 +4890,7 @@
         <v>64</v>
       </c>
       <c r="AR30" s="8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AS30" s="8" t="s">
         <v>67</v>
@@ -4884,7 +4902,7 @@
     <row r="31" ht="18.75" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A31" s="7"/>
       <c r="B31" s="8" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C31" s="8" t="s">
         <v>48</v>
@@ -4923,7 +4941,7 @@
         <v>54</v>
       </c>
       <c r="O31" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="P31" s="8" t="s">
         <v>56</v>
@@ -5001,7 +5019,7 @@
         <v>63</v>
       </c>
       <c r="AO31" s="8" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="AP31" s="8" t="s">
         <v>64</v>
@@ -5010,7 +5028,7 @@
         <v>64</v>
       </c>
       <c r="AR31" s="8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AS31" s="8" t="s">
         <v>67</v>
@@ -5022,7 +5040,7 @@
     <row r="32" ht="18.75" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A32" s="7"/>
       <c r="B32" s="8" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C32" s="8" t="s">
         <v>48</v>
@@ -5061,7 +5079,7 @@
         <v>54</v>
       </c>
       <c r="O32" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="P32" s="8" t="s">
         <v>56</v>
@@ -5148,7 +5166,7 @@
         <v>64</v>
       </c>
       <c r="AR32" s="8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AS32" s="8" t="s">
         <v>67</v>
@@ -5160,7 +5178,7 @@
     <row r="33" ht="18.75" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A33" s="7"/>
       <c r="B33" s="8" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C33" s="8" t="s">
         <v>48</v>
@@ -5199,7 +5217,7 @@
         <v>54</v>
       </c>
       <c r="O33" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="P33" s="8" t="s">
         <v>56</v>
@@ -5277,7 +5295,7 @@
         <v>63</v>
       </c>
       <c r="AO33" s="8" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="AP33" s="8" t="s">
         <v>65</v>
@@ -5286,7 +5304,7 @@
         <v>64</v>
       </c>
       <c r="AR33" s="8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AS33" s="8" t="s">
         <v>67</v>

</xml_diff>

<commit_message>
Scenario sheet: add POL-3GW-CT, drop unused gas rows
- POL-3GW now has no carbon tax; new POL-3GW-CT row carries CT_2050
- Remove REN-LIMIT, REN-PUSH, GAS-LATE, POL6-*, POL-6GW_DUP; renumber rows
- run_scenario set to 0 on REF-LC and P0/P1 rows; show/export filled in

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scenarios/Coal_Flexibilisation/scenarios_to_run.xlsx
+++ b/scenarios/Coal_Flexibilisation/scenarios_to_run.xlsx
@@ -1,17 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30527"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D52F6273-2630-43A7-B37C-C71F03D43635}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="scenario_definition" state="visible" r:id="rId4"/>
+    <sheet name="scenario_definition" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1088" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="959" uniqueCount="197">
   <si>
     <t>index</t>
   </si>
@@ -220,51 +237,42 @@
     <t>BASE2</t>
   </si>
   <si>
-    <t>POL-2GW</t>
-  </si>
-  <si>
-    <t>2025, 2030, 2035, 2040, 2045, 2051</t>
+    <t>POL-3GW</t>
+  </si>
+  <si>
+    <t>3GW_GAS</t>
+  </si>
+  <si>
+    <t>POL-3GW-CT</t>
+  </si>
+  <si>
+    <t>POL-6GW</t>
+  </si>
+  <si>
+    <t>6GW_GAS</t>
+  </si>
+  <si>
+    <t>POL-18.25GW</t>
+  </si>
+  <si>
+    <t>IRP25_GAS</t>
+  </si>
+  <si>
+    <t>COAL-FAST</t>
+  </si>
+  <si>
+    <t>2025, 2030, 2035, 2040, 2045, 2054</t>
   </si>
   <si>
     <t>NO_MIN_GAS</t>
   </si>
   <si>
-    <t>POL-6GW</t>
-  </si>
-  <si>
-    <t>2025, 2030, 2035, 2040, 2045, 2052</t>
-  </si>
-  <si>
-    <t>POL-16GW</t>
-  </si>
-  <si>
-    <t>2025, 2030, 2035, 2040, 2045, 2053</t>
-  </si>
-  <si>
-    <t>COAL-FAST</t>
-  </si>
-  <si>
-    <t>2025, 2030, 2035, 2040, 2045, 2054</t>
-  </si>
-  <si>
     <t>COAL-SLOW</t>
   </si>
   <si>
     <t>2025, 2030, 2035, 2040, 2045, 2055</t>
   </si>
   <si>
-    <t>REN-LIMIT</t>
-  </si>
-  <si>
-    <t>2025, 2030, 2035, 2040, 2045, 2056</t>
-  </si>
-  <si>
-    <t>REN-PUSH</t>
-  </si>
-  <si>
-    <t>2025, 2030, 2035, 2040, 2045, 2057</t>
-  </si>
-  <si>
     <t>DEM-CENTRAL</t>
   </si>
   <si>
@@ -313,27 +321,6 @@
     <t>2025, 2030, 2035, 2040, 2045, 2065</t>
   </si>
   <si>
-    <t>GAS-LATE</t>
-  </si>
-  <si>
-    <t>2025, 2030, 2035, 2040, 2045, 2066</t>
-  </si>
-  <si>
-    <t>POL6-COAL-SLOW</t>
-  </si>
-  <si>
-    <t>2025, 2030, 2035, 2040, 2045, 2067</t>
-  </si>
-  <si>
-    <t>POL6-REN-PUSH</t>
-  </si>
-  <si>
-    <t>2025, 2030, 2035, 2040, 2045, 2068</t>
-  </si>
-  <si>
-    <t>2025, 2030, 2035, 2040, 2045, 2069</t>
-  </si>
-  <si>
     <t>* Solver used to solve the LP optimization problem.</t>
   </si>
   <si>
@@ -629,28 +616,31 @@
   </si>
   <si>
     <t>P1_CT_R</t>
+  </si>
+  <si>
+    <t>REF-LC-CT</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <color rgb="FF3F3F3F"/>
       <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
       <color rgb="FF000000"/>
-      <sz val="11"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -1086,52 +1076,51 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AT33"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:AT30"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.285714285714286" customWidth="1"/>
-    <col min="2" max="2" width="26.285714285714285" customWidth="1"/>
-    <col min="3" max="7" width="9.285714285714286" customWidth="1"/>
-    <col min="8" max="8" width="11.285714285714286" customWidth="1"/>
-    <col min="9" max="9" width="32.285714285714285" customWidth="1"/>
-    <col min="10" max="10" width="15.857142857142858" customWidth="1"/>
-    <col min="11" max="12" width="9.285714285714286" customWidth="1"/>
-    <col min="13" max="13" width="18.142857142857142" customWidth="1"/>
-    <col min="14" max="14" width="14.571428571428571" customWidth="1"/>
-    <col min="15" max="15" width="15.142857142857142" customWidth="1"/>
-    <col min="16" max="16" width="12.857142857142858" customWidth="1"/>
+    <col min="1" max="1" width="9.33203125" customWidth="1"/>
+    <col min="2" max="2" width="26.33203125" customWidth="1"/>
+    <col min="3" max="7" width="9.33203125" customWidth="1"/>
+    <col min="8" max="8" width="11.33203125" customWidth="1"/>
+    <col min="9" max="9" width="32.33203125" customWidth="1"/>
+    <col min="10" max="10" width="15.88671875" customWidth="1"/>
+    <col min="11" max="12" width="9.33203125" customWidth="1"/>
+    <col min="13" max="13" width="18.109375" customWidth="1"/>
+    <col min="14" max="14" width="14.5546875" customWidth="1"/>
+    <col min="15" max="15" width="15.109375" customWidth="1"/>
+    <col min="16" max="16" width="12.88671875" customWidth="1"/>
     <col min="17" max="17" width="14" customWidth="1"/>
-    <col min="18" max="18" width="28.285714285714285" customWidth="1"/>
+    <col min="18" max="18" width="28.33203125" customWidth="1"/>
     <col min="19" max="19" width="11" customWidth="1"/>
-    <col min="20" max="20" width="25.285714285714285" customWidth="1"/>
+    <col min="20" max="20" width="25.33203125" customWidth="1"/>
     <col min="21" max="22" width="14" customWidth="1"/>
-    <col min="23" max="23" width="14.142857142857142" customWidth="1"/>
-    <col min="24" max="24" width="10.714285714285714" customWidth="1"/>
-    <col min="25" max="25" width="11.142857142857142" customWidth="1"/>
-    <col min="26" max="26" width="12.285714285714286" customWidth="1"/>
-    <col min="27" max="27" width="11.571428571428571" customWidth="1"/>
-    <col min="28" max="28" width="12.285714285714286" customWidth="1"/>
-    <col min="29" max="29" width="11.571428571428571" customWidth="1"/>
-    <col min="30" max="30" width="17.428571428571427" customWidth="1"/>
-    <col min="31" max="31" width="12.428571428571429" customWidth="1"/>
-    <col min="32" max="32" width="12.857142857142858" customWidth="1"/>
-    <col min="33" max="34" width="12.428571428571429" customWidth="1"/>
-    <col min="35" max="35" width="12.142857142857142" customWidth="1"/>
-    <col min="36" max="36" width="12.857142857142858" customWidth="1"/>
+    <col min="23" max="23" width="14.109375" customWidth="1"/>
+    <col min="24" max="24" width="10.6640625" customWidth="1"/>
+    <col min="25" max="25" width="11.109375" customWidth="1"/>
+    <col min="26" max="26" width="12.33203125" customWidth="1"/>
+    <col min="27" max="27" width="11.5546875" customWidth="1"/>
+    <col min="28" max="28" width="12.33203125" customWidth="1"/>
+    <col min="29" max="29" width="11.5546875" customWidth="1"/>
+    <col min="30" max="30" width="17.44140625" customWidth="1"/>
+    <col min="31" max="31" width="12.44140625" customWidth="1"/>
+    <col min="32" max="32" width="12.88671875" customWidth="1"/>
+    <col min="33" max="34" width="12.44140625" customWidth="1"/>
+    <col min="35" max="35" width="12.109375" customWidth="1"/>
+    <col min="36" max="36" width="12.88671875" customWidth="1"/>
     <col min="37" max="37" width="13" customWidth="1"/>
-    <col min="38" max="38" width="18.857142857142858" customWidth="1"/>
-    <col min="39" max="39" width="9.285714285714286" customWidth="1"/>
+    <col min="38" max="38" width="18.88671875" customWidth="1"/>
+    <col min="39" max="39" width="9.33203125" customWidth="1"/>
     <col min="40" max="40" width="10" customWidth="1"/>
     <col min="41" max="41" width="13" customWidth="1"/>
-    <col min="42" max="43" width="9.285714285714286" customWidth="1"/>
-    <col min="44" max="44" width="15.571428571428571" customWidth="1"/>
-    <col min="45" max="45" width="15.428571428571429" customWidth="1"/>
-    <col min="46" max="46" width="15.857142857142858" customWidth="1"/>
-    <col min="47" max="92" width="13.571428571428571" customWidth="1"/>
+    <col min="42" max="43" width="9.33203125" customWidth="1"/>
+    <col min="44" max="44" width="15.5546875" customWidth="1"/>
+    <col min="45" max="45" width="15.44140625" customWidth="1"/>
+    <col min="46" max="46" width="15.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32.25" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:46" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1271,7 +1260,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>46</v>
       </c>
@@ -1281,17 +1270,17 @@
       <c r="C2" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="D2" s="7">
-        <f>TRUE()</f>
-      </c>
-      <c r="E2" s="7">
-        <f>TRUE()</f>
+      <c r="D2" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>49</v>
       </c>
       <c r="F2" s="7">
         <v>0</v>
       </c>
-      <c r="G2" s="7" t="s">
-        <v>49</v>
+      <c r="G2" s="7">
+        <v>0</v>
       </c>
       <c r="H2" s="7">
         <v>1</v>
@@ -1357,7 +1346,7 @@
         <v>57</v>
       </c>
       <c r="AC2" s="7">
-        <v>0.092</v>
+        <v>9.1999999999999998E-2</v>
       </c>
       <c r="AD2" s="8" t="s">
         <v>57</v>
@@ -1396,7 +1385,7 @@
         <v>64</v>
       </c>
       <c r="AP2" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AQ2" s="8" t="s">
         <v>64</v>
@@ -1411,21 +1400,25 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A3" s="7">
         <v>2</v>
       </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>POL-3GW</t>
-        </is>
+      <c r="B3" s="8" t="s">
+        <v>196</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
+      <c r="D3" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="F3" s="7">
+        <v>0</v>
+      </c>
       <c r="G3" s="7">
         <v>0</v>
       </c>
@@ -1493,7 +1486,7 @@
         <v>57</v>
       </c>
       <c r="AC3" s="7">
-        <v>0.092</v>
+        <v>9.1999999999999998E-2</v>
       </c>
       <c r="AD3" s="8" t="s">
         <v>57</v>
@@ -1510,10 +1503,8 @@
       <c r="AH3" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="AI3" s="8" t="inlineStr">
-        <is>
-          <t>3GW_GAS</t>
-        </is>
+      <c r="AI3" s="8" t="s">
+        <v>60</v>
       </c>
       <c r="AJ3" s="8" t="s">
         <v>61</v>
@@ -1549,19 +1540,25 @@
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A4" s="7">
         <v>3</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
+      <c r="D4" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="F4" s="7">
+        <v>0</v>
+      </c>
       <c r="G4" s="7">
         <v>0</v>
       </c>
@@ -1629,7 +1626,7 @@
         <v>57</v>
       </c>
       <c r="AC4" s="7">
-        <v>0.092</v>
+        <v>9.1999999999999998E-2</v>
       </c>
       <c r="AD4" s="8" t="s">
         <v>57</v>
@@ -1646,10 +1643,8 @@
       <c r="AH4" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="AI4" s="8" t="inlineStr">
-        <is>
-          <t>6GW_GAS</t>
-        </is>
+      <c r="AI4" s="8" t="s">
+        <v>70</v>
       </c>
       <c r="AJ4" s="8" t="s">
         <v>61</v>
@@ -1670,7 +1665,7 @@
         <v>64</v>
       </c>
       <c r="AP4" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AQ4" s="8" t="s">
         <v>64</v>
@@ -1685,21 +1680,25 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A5" s="7">
         <v>4</v>
       </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>POL-18.25GW</t>
-        </is>
+      <c r="B5" s="8" t="s">
+        <v>71</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
+      <c r="D5" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="F5" s="7">
+        <v>0</v>
+      </c>
       <c r="G5" s="7">
         <v>0</v>
       </c>
@@ -1767,7 +1766,7 @@
         <v>57</v>
       </c>
       <c r="AC5" s="7">
-        <v>0.092</v>
+        <v>9.1999999999999998E-2</v>
       </c>
       <c r="AD5" s="8" t="s">
         <v>57</v>
@@ -1784,10 +1783,8 @@
       <c r="AH5" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="AI5" s="8" t="inlineStr">
-        <is>
-          <t>IRP25_GAS</t>
-        </is>
+      <c r="AI5" s="8" t="s">
+        <v>70</v>
       </c>
       <c r="AJ5" s="8" t="s">
         <v>61</v>
@@ -1823,144 +1820,12 @@
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:46" x14ac:dyDescent="0.25">
-      <c r="A6" s="7">
-        <v>5</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7">
-        <v>1</v>
-      </c>
-      <c r="I6" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="J6" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="K6" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="L6" s="7">
-        <v>1</v>
-      </c>
-      <c r="M6" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="N6" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="O6" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="P6" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="Q6" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="R6" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="S6" s="7">
-        <v>1</v>
-      </c>
-      <c r="T6" s="7">
-        <v>1</v>
-      </c>
-      <c r="U6" s="10">
-        <v>0.65</v>
-      </c>
-      <c r="V6" s="7">
-        <v>1</v>
-      </c>
-      <c r="W6" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="X6" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="Y6" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="Z6" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AA6" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AB6" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="AC6" s="7">
-        <v>0.092</v>
-      </c>
-      <c r="AD6" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="AE6" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AF6" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AG6" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AH6" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AI6" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AJ6" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="AK6" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL6" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AM6" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AN6" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="AO6" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="AP6" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="AQ6" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="AR6" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="AS6" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="AT6" s="8" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="7" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A7" s="7">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>48</v>
@@ -1973,7 +1838,7 @@
         <v>1</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="J7" s="8" t="s">
         <v>51</v>
@@ -2033,7 +1898,7 @@
         <v>57</v>
       </c>
       <c r="AC7" s="7">
-        <v>0.092</v>
+        <v>9.1999999999999998E-2</v>
       </c>
       <c r="AD7" s="8" t="s">
         <v>57</v>
@@ -2051,13 +1916,13 @@
         <v>60</v>
       </c>
       <c r="AI7" s="8" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="AJ7" s="8" t="s">
         <v>61</v>
       </c>
       <c r="AK7" s="8" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="AL7" s="8" t="s">
         <v>59</v>
@@ -2087,12 +1952,12 @@
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A8" s="7">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>48</v>
@@ -2105,7 +1970,7 @@
         <v>1</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>81</v>
+        <v>50</v>
       </c>
       <c r="J8" s="8" t="s">
         <v>51</v>
@@ -2165,7 +2030,7 @@
         <v>57</v>
       </c>
       <c r="AC8" s="7">
-        <v>0.092</v>
+        <v>9.1999999999999998E-2</v>
       </c>
       <c r="AD8" s="8" t="s">
         <v>57</v>
@@ -2183,13 +2048,13 @@
         <v>60</v>
       </c>
       <c r="AI8" s="8" t="s">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="AJ8" s="8" t="s">
         <v>61</v>
       </c>
       <c r="AK8" s="8" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="AL8" s="8" t="s">
         <v>59</v>
@@ -2219,12 +2084,12 @@
         <v>68</v>
       </c>
     </row>
-    <row r="9" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A9" s="7">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>48</v>
@@ -2237,7 +2102,7 @@
         <v>1</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="J9" s="8" t="s">
         <v>51</v>
@@ -2297,7 +2162,7 @@
         <v>57</v>
       </c>
       <c r="AC9" s="7">
-        <v>0.092</v>
+        <v>9.1999999999999998E-2</v>
       </c>
       <c r="AD9" s="8" t="s">
         <v>57</v>
@@ -2321,7 +2186,7 @@
         <v>61</v>
       </c>
       <c r="AK9" s="8" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="AL9" s="8" t="s">
         <v>59</v>
@@ -2351,12 +2216,12 @@
         <v>68</v>
       </c>
     </row>
-    <row r="10" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A10" s="7">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="C10" s="8" t="s">
         <v>48</v>
@@ -2369,7 +2234,7 @@
         <v>1</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="J10" s="8" t="s">
         <v>51</v>
@@ -2429,7 +2294,7 @@
         <v>57</v>
       </c>
       <c r="AC10" s="7">
-        <v>0.092</v>
+        <v>9.1999999999999998E-2</v>
       </c>
       <c r="AD10" s="8" t="s">
         <v>57</v>
@@ -2453,7 +2318,7 @@
         <v>61</v>
       </c>
       <c r="AK10" s="8" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="AL10" s="8" t="s">
         <v>59</v>
@@ -2483,12 +2348,12 @@
         <v>68</v>
       </c>
     </row>
-    <row r="11" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A11" s="7">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>48</v>
@@ -2501,7 +2366,7 @@
         <v>1</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="J11" s="8" t="s">
         <v>51</v>
@@ -2561,7 +2426,7 @@
         <v>57</v>
       </c>
       <c r="AC11" s="7">
-        <v>0.092</v>
+        <v>9.1999999999999998E-2</v>
       </c>
       <c r="AD11" s="8" t="s">
         <v>57</v>
@@ -2585,7 +2450,7 @@
         <v>61</v>
       </c>
       <c r="AK11" s="8" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="AL11" s="8" t="s">
         <v>59</v>
@@ -2615,12 +2480,12 @@
         <v>68</v>
       </c>
     </row>
-    <row r="12" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A12" s="7">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>48</v>
@@ -2633,7 +2498,7 @@
         <v>1</v>
       </c>
       <c r="I12" s="8" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="J12" s="8" t="s">
         <v>51</v>
@@ -2693,7 +2558,7 @@
         <v>57</v>
       </c>
       <c r="AC12" s="7">
-        <v>0.092</v>
+        <v>9.1999999999999998E-2</v>
       </c>
       <c r="AD12" s="8" t="s">
         <v>57</v>
@@ -2717,7 +2582,7 @@
         <v>61</v>
       </c>
       <c r="AK12" s="8" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="AL12" s="8" t="s">
         <v>59</v>
@@ -2747,12 +2612,12 @@
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A13" s="7">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>48</v>
@@ -2765,7 +2630,7 @@
         <v>1</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="J13" s="8" t="s">
         <v>51</v>
@@ -2825,7 +2690,7 @@
         <v>57</v>
       </c>
       <c r="AC13" s="7">
-        <v>0.092</v>
+        <v>9.1999999999999998E-2</v>
       </c>
       <c r="AD13" s="8" t="s">
         <v>57</v>
@@ -2849,7 +2714,7 @@
         <v>61</v>
       </c>
       <c r="AK13" s="8" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="AL13" s="8" t="s">
         <v>59</v>
@@ -2879,12 +2744,12 @@
         <v>68</v>
       </c>
     </row>
-    <row r="14" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A14" s="7">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>48</v>
@@ -2897,7 +2762,7 @@
         <v>1</v>
       </c>
       <c r="I14" s="8" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="J14" s="8" t="s">
         <v>51</v>
@@ -2957,7 +2822,7 @@
         <v>57</v>
       </c>
       <c r="AC14" s="7">
-        <v>0.092</v>
+        <v>9.1999999999999998E-2</v>
       </c>
       <c r="AD14" s="8" t="s">
         <v>57</v>
@@ -2981,7 +2846,7 @@
         <v>61</v>
       </c>
       <c r="AK14" s="8" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="AL14" s="8" t="s">
         <v>59</v>
@@ -3011,12 +2876,12 @@
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A15" s="7">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C15" s="8" t="s">
         <v>48</v>
@@ -3029,7 +2894,7 @@
         <v>1</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="J15" s="8" t="s">
         <v>51</v>
@@ -3089,7 +2954,7 @@
         <v>57</v>
       </c>
       <c r="AC15" s="7">
-        <v>0.092</v>
+        <v>9.1999999999999998E-2</v>
       </c>
       <c r="AD15" s="8" t="s">
         <v>57</v>
@@ -3113,7 +2978,7 @@
         <v>61</v>
       </c>
       <c r="AK15" s="8" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="AL15" s="8" t="s">
         <v>59</v>
@@ -3143,12 +3008,12 @@
         <v>68</v>
       </c>
     </row>
-    <row r="16" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A16" s="7">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="C16" s="8" t="s">
         <v>48</v>
@@ -3161,7 +3026,7 @@
         <v>1</v>
       </c>
       <c r="I16" s="8" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="J16" s="8" t="s">
         <v>51</v>
@@ -3221,7 +3086,7 @@
         <v>57</v>
       </c>
       <c r="AC16" s="7">
-        <v>0.092</v>
+        <v>9.1999999999999998E-2</v>
       </c>
       <c r="AD16" s="8" t="s">
         <v>57</v>
@@ -3245,7 +3110,7 @@
         <v>61</v>
       </c>
       <c r="AK16" s="8" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="AL16" s="8" t="s">
         <v>59</v>
@@ -3275,12 +3140,12 @@
         <v>68</v>
       </c>
     </row>
-    <row r="17" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A17" s="7">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C17" s="8" t="s">
         <v>48</v>
@@ -3293,7 +3158,7 @@
         <v>1</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="J17" s="8" t="s">
         <v>51</v>
@@ -3353,7 +3218,7 @@
         <v>57</v>
       </c>
       <c r="AC17" s="7">
-        <v>0.092</v>
+        <v>9.1999999999999998E-2</v>
       </c>
       <c r="AD17" s="8" t="s">
         <v>57</v>
@@ -3377,7 +3242,7 @@
         <v>61</v>
       </c>
       <c r="AK17" s="8" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="AL17" s="8" t="s">
         <v>59</v>
@@ -3407,12 +3272,12 @@
         <v>68</v>
       </c>
     </row>
-    <row r="18" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A18" s="7">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C18" s="8" t="s">
         <v>48</v>
@@ -3425,7 +3290,7 @@
         <v>1</v>
       </c>
       <c r="I18" s="8" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="J18" s="8" t="s">
         <v>51</v>
@@ -3485,7 +3350,7 @@
         <v>57</v>
       </c>
       <c r="AC18" s="7">
-        <v>0.092</v>
+        <v>9.1999999999999998E-2</v>
       </c>
       <c r="AD18" s="8" t="s">
         <v>57</v>
@@ -3509,7 +3374,7 @@
         <v>61</v>
       </c>
       <c r="AK18" s="8" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="AL18" s="8" t="s">
         <v>59</v>
@@ -3539,701 +3404,726 @@
         <v>68</v>
       </c>
     </row>
-    <row r="19" spans="1:46" x14ac:dyDescent="0.25">
-      <c r="A19" s="7">
-        <v>18</v>
-      </c>
-      <c r="B19" s="8" t="s">
+    <row r="20" spans="1:46" ht="362.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="12"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="E20" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="G20" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="H20" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="I20" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="J20" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="K20" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="L20" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="M20" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="N20" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="O20" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="P20" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="Q20" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="R20" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="S20" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="T20" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="U20" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="V20" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="W20" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="X20" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="Y20" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="Z20" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="AA20" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="AB20" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="AC20" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="AD20" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="AE20" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="AF20" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="AG20" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="AH20" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="AI20" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="AJ20" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="AK20" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="AL20" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="AM20" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="AN20" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="AO20" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="AP20" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="AQ20" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="AR20" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="AS20" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="AT20" s="14" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="21" spans="1:46" ht="252" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="16"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="F21" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="H21" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="I21" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="J21" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="K21" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="L21" s="14" t="s">
+        <v>148</v>
+      </c>
+      <c r="M21" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="N21" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="O21" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="P21" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="Q21" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="R21" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="S21" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="T21" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="U21" s="14" t="s">
+        <v>157</v>
+      </c>
+      <c r="V21" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="W21" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="X21" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="Y21" s="14" t="s">
+        <v>161</v>
+      </c>
+      <c r="Z21" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="AA21" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="AB21" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="AC21" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="AD21" s="14" t="s">
+        <v>166</v>
+      </c>
+      <c r="AE21" s="14" t="s">
+        <v>167</v>
+      </c>
+      <c r="AF21" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="AG21" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="AH21" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="AI21" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="AJ21" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="AK21" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="AL21" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="AM21" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AN21" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="AO21" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AP21" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="AQ21" s="14"/>
+      <c r="AR21" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="AS21" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="AT21" s="14" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="23" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="7"/>
+      <c r="B23" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="C23" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="7"/>
-      <c r="H19" s="7">
-        <v>1</v>
-      </c>
-      <c r="I19" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="J19" s="8" t="s">
+      <c r="D23" s="7" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="E23" s="7" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="F23" s="7">
+        <v>0</v>
+      </c>
+      <c r="G23" s="18" t="s">
+        <v>183</v>
+      </c>
+      <c r="H23" s="7">
+        <v>1</v>
+      </c>
+      <c r="I23" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="J23" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="K19" s="8" t="s">
+      <c r="K23" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="L19" s="7">
-        <v>1</v>
-      </c>
-      <c r="M19" s="8" t="s">
+      <c r="L23" s="7">
+        <v>10</v>
+      </c>
+      <c r="M23" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="N19" s="8" t="s">
+      <c r="N23" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="O19" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="P19" s="8" t="s">
+      <c r="O23" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="P23" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="Q19" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="R19" s="8" t="s">
+      <c r="Q23" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="R23" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="S19" s="7">
-        <v>1</v>
-      </c>
-      <c r="T19" s="7">
-        <v>1</v>
-      </c>
-      <c r="U19" s="10">
+      <c r="S23" s="7">
+        <v>1</v>
+      </c>
+      <c r="T23" s="7">
+        <v>1</v>
+      </c>
+      <c r="U23" s="10">
         <v>0.65</v>
       </c>
-      <c r="V19" s="7">
-        <v>1</v>
-      </c>
-      <c r="W19" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="X19" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="Y19" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="Z19" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AA19" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AB19" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="AC19" s="7">
-        <v>0.092</v>
-      </c>
-      <c r="AD19" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="AE19" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AF19" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AG19" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AH19" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AI19" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AJ19" s="8" t="s">
+      <c r="V23" s="7">
+        <v>1</v>
+      </c>
+      <c r="W23" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="X23" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="Y23" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="Z23" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="AA23" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="AB23" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="AC23" s="7">
+        <v>9.1999999999999998E-2</v>
+      </c>
+      <c r="AD23" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="AE23" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="AF23" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG23" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="AH23" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="AI23" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="AJ23" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="AK19" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL19" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AM19" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AN19" s="8" t="s">
+      <c r="AK23" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="AL23" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="AM23" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="AN23" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="AO19" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="AP19" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="AQ19" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="AR19" s="11" t="s">
+      <c r="AO23" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="AP23" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="AQ23" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="AR23" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="AS19" s="8" t="s">
+      <c r="AS23" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="AT19" s="8" t="s">
+      <c r="AT23" s="8" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="20" spans="1:46" x14ac:dyDescent="0.25">
-      <c r="A20" s="7">
-        <v>19</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="C20" s="8" t="s">
+    <row r="24" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="7"/>
+      <c r="B24" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="C24" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="7"/>
-      <c r="H20" s="7">
-        <v>1</v>
-      </c>
-      <c r="I20" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="J20" s="8" t="s">
+      <c r="D24" s="7" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="E24" s="7" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="F24" s="7">
+        <v>0</v>
+      </c>
+      <c r="G24" s="7" t="b">
+        <f>FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H24" s="7">
+        <v>1</v>
+      </c>
+      <c r="I24" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="J24" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="K20" s="8" t="s">
+      <c r="K24" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="L20" s="7">
-        <v>1</v>
-      </c>
-      <c r="M20" s="8" t="s">
+      <c r="L24" s="7">
+        <v>10</v>
+      </c>
+      <c r="M24" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="N20" s="8" t="s">
+      <c r="N24" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="O20" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="P20" s="8" t="s">
+      <c r="O24" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="P24" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="Q20" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="R20" s="8" t="s">
+      <c r="Q24" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="R24" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="S20" s="7">
-        <v>1</v>
-      </c>
-      <c r="T20" s="7">
-        <v>1</v>
-      </c>
-      <c r="U20" s="10">
+      <c r="S24" s="7">
+        <v>1</v>
+      </c>
+      <c r="T24" s="7">
+        <v>1</v>
+      </c>
+      <c r="U24" s="10">
         <v>0.65</v>
       </c>
-      <c r="V20" s="7">
-        <v>1</v>
-      </c>
-      <c r="W20" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="X20" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="Y20" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="Z20" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AA20" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AB20" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="AC20" s="7">
-        <v>0.092</v>
-      </c>
-      <c r="AD20" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="AE20" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AF20" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AG20" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AH20" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AI20" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AJ20" s="8" t="s">
+      <c r="V24" s="7">
+        <v>1</v>
+      </c>
+      <c r="W24" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="X24" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="Y24" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="Z24" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="AA24" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="AB24" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="AC24" s="7">
+        <v>9.1999999999999998E-2</v>
+      </c>
+      <c r="AD24" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="AE24" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="AF24" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG24" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="AH24" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="AI24" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="AJ24" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="AK20" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL20" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AM20" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AN20" s="8" t="s">
+      <c r="AK24" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="AL24" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="AM24" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="AN24" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="AO20" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="AP20" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="AQ20" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="AR20" s="11" t="s">
+      <c r="AO24" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="AP24" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="AQ24" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="AR24" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="AS20" s="8" t="s">
+      <c r="AS24" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="AT20" s="8" t="s">
+      <c r="AT24" s="8" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="21" spans="1:46" x14ac:dyDescent="0.25">
-      <c r="A21" s="7">
-        <v>20</v>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>POL-6GW_DUP</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="s">
+    <row r="25" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="7"/>
+      <c r="B25" s="8" t="s">
+        <v>188</v>
+      </c>
+      <c r="C25" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7">
+      <c r="D25" s="7" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="E25" s="7" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="F25" s="7">
         <v>0</v>
       </c>
-      <c r="H21" s="7">
-        <v>1</v>
-      </c>
-      <c r="I21" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="J21" s="8" t="s">
+      <c r="G25" s="7" t="b">
+        <f>FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="H25" s="7">
+        <v>1</v>
+      </c>
+      <c r="I25" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="J25" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="K21" s="8" t="s">
+      <c r="K25" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="L21" s="7">
-        <v>1</v>
-      </c>
-      <c r="M21" s="8" t="s">
+      <c r="L25" s="7">
+        <v>10</v>
+      </c>
+      <c r="M25" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="N21" s="8" t="s">
+      <c r="N25" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="O21" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="P21" s="8" t="s">
+      <c r="O25" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="P25" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="Q21" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="R21" s="8" t="s">
+      <c r="Q25" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="R25" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="S21" s="7">
-        <v>1</v>
-      </c>
-      <c r="T21" s="7">
-        <v>1</v>
-      </c>
-      <c r="U21" s="10">
+      <c r="S25" s="7">
+        <v>1</v>
+      </c>
+      <c r="T25" s="7">
+        <v>1</v>
+      </c>
+      <c r="U25" s="10">
         <v>0.65</v>
       </c>
-      <c r="V21" s="7">
-        <v>1</v>
-      </c>
-      <c r="W21" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="X21" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="Y21" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="Z21" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AA21" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AB21" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="AC21" s="7">
-        <v>0.092</v>
-      </c>
-      <c r="AD21" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="AE21" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AF21" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AG21" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AH21" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AI21" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AJ21" s="8" t="s">
+      <c r="V25" s="7">
+        <v>1</v>
+      </c>
+      <c r="W25" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="X25" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="Y25" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="Z25" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="AA25" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="AB25" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="AC25" s="7">
+        <v>9.1999999999999998E-2</v>
+      </c>
+      <c r="AD25" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="AE25" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="AF25" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG25" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="AH25" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="AI25" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="AJ25" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="AK21" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL21" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AM21" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AN21" s="8" t="s">
+      <c r="AK25" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="AL25" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="AM25" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="AN25" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="AO21" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="AP21" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="AQ21" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="AR21" s="11" t="s">
+      <c r="AO25" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="AP25" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="AQ25" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="AR25" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="AS21" s="8" t="s">
+      <c r="AS25" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="AT21" s="8" t="s">
+      <c r="AT25" s="8" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="23" ht="453" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
-      <c r="A23" s="12"/>
-      <c r="B23" s="13"/>
-      <c r="C23" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="D23" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="E23" s="14" t="s">
-        <v>109</v>
-      </c>
-      <c r="F23" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="G23" s="14" t="s">
-        <v>111</v>
-      </c>
-      <c r="H23" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="I23" s="14" t="s">
-        <v>113</v>
-      </c>
-      <c r="J23" s="14" t="s">
-        <v>114</v>
-      </c>
-      <c r="K23" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="L23" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="M23" s="14" t="s">
-        <v>117</v>
-      </c>
-      <c r="N23" s="14" t="s">
-        <v>118</v>
-      </c>
-      <c r="O23" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="P23" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="Q23" s="14" t="s">
-        <v>121</v>
-      </c>
-      <c r="R23" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="S23" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="T23" s="12" t="s">
-        <v>124</v>
-      </c>
-      <c r="U23" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="V23" s="15" t="s">
-        <v>126</v>
-      </c>
-      <c r="W23" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="X23" s="14" t="s">
-        <v>128</v>
-      </c>
-      <c r="Y23" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="Z23" s="14" t="s">
-        <v>130</v>
-      </c>
-      <c r="AA23" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="AB23" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="AC23" s="15" t="s">
-        <v>133</v>
-      </c>
-      <c r="AD23" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="AE23" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="AF23" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="AG23" s="14" t="s">
-        <v>137</v>
-      </c>
-      <c r="AH23" s="14" t="s">
-        <v>138</v>
-      </c>
-      <c r="AI23" s="14" t="s">
-        <v>139</v>
-      </c>
-      <c r="AJ23" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="AK23" s="14" t="s">
-        <v>141</v>
-      </c>
-      <c r="AL23" s="14" t="s">
-        <v>142</v>
-      </c>
-      <c r="AM23" s="14" t="s">
-        <v>143</v>
-      </c>
-      <c r="AN23" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="AO23" s="14" t="s">
-        <v>145</v>
-      </c>
-      <c r="AP23" s="14" t="s">
-        <v>146</v>
-      </c>
-      <c r="AQ23" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="AR23" s="14" t="s">
-        <v>148</v>
-      </c>
-      <c r="AS23" s="14" t="s">
-        <v>149</v>
-      </c>
-      <c r="AT23" s="14" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="24" ht="315" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
-      <c r="A24" s="16"/>
-      <c r="B24" s="17"/>
-      <c r="C24" s="14" t="s">
-        <v>151</v>
-      </c>
-      <c r="D24" s="14" t="s">
-        <v>152</v>
-      </c>
-      <c r="E24" s="14" t="s">
-        <v>152</v>
-      </c>
-      <c r="F24" s="14" t="s">
-        <v>152</v>
-      </c>
-      <c r="G24" s="14" t="s">
-        <v>153</v>
-      </c>
-      <c r="H24" s="14" t="s">
-        <v>154</v>
-      </c>
-      <c r="I24" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="J24" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="K24" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="L24" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="M24" s="14" t="s">
-        <v>159</v>
-      </c>
-      <c r="N24" s="14" t="s">
-        <v>160</v>
-      </c>
-      <c r="O24" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="P24" s="14" t="s">
-        <v>162</v>
-      </c>
-      <c r="Q24" s="14" t="s">
-        <v>163</v>
-      </c>
-      <c r="R24" s="14" t="s">
-        <v>164</v>
-      </c>
-      <c r="S24" s="14" t="s">
-        <v>165</v>
-      </c>
-      <c r="T24" s="14" t="s">
-        <v>166</v>
-      </c>
-      <c r="U24" s="14" t="s">
-        <v>167</v>
-      </c>
-      <c r="V24" s="14" t="s">
-        <v>168</v>
-      </c>
-      <c r="W24" s="14" t="s">
-        <v>169</v>
-      </c>
-      <c r="X24" s="14" t="s">
-        <v>170</v>
-      </c>
-      <c r="Y24" s="14" t="s">
-        <v>171</v>
-      </c>
-      <c r="Z24" s="14" t="s">
-        <v>172</v>
-      </c>
-      <c r="AA24" s="14" t="s">
-        <v>173</v>
-      </c>
-      <c r="AB24" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="AC24" s="14" t="s">
-        <v>175</v>
-      </c>
-      <c r="AD24" s="14" t="s">
-        <v>176</v>
-      </c>
-      <c r="AE24" s="14" t="s">
-        <v>177</v>
-      </c>
-      <c r="AF24" s="14" t="s">
-        <v>178</v>
-      </c>
-      <c r="AG24" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AH24" s="14" t="s">
-        <v>180</v>
-      </c>
-      <c r="AI24" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="AJ24" s="14" t="s">
-        <v>182</v>
-      </c>
-      <c r="AK24" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="AL24" s="14" t="s">
-        <v>184</v>
-      </c>
-      <c r="AM24" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AN24" s="14" t="s">
-        <v>186</v>
-      </c>
-      <c r="AO24" s="14" t="s">
-        <v>187</v>
-      </c>
-      <c r="AP24" s="14" t="s">
-        <v>188</v>
-      </c>
-      <c r="AQ24" s="14"/>
-      <c r="AR24" s="14" t="s">
-        <v>189</v>
-      </c>
-      <c r="AS24" s="14" t="s">
-        <v>190</v>
-      </c>
-      <c r="AT24" s="14" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="26" ht="18.75" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="7"/>
       <c r="B26" s="8" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C26" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="D26" s="7">
+      <c r="D26" s="7" t="b">
         <f>TRUE()</f>
-      </c>
-      <c r="E26" s="7">
+        <v>1</v>
+      </c>
+      <c r="E26" s="7" t="b">
         <f>TRUE()</f>
+        <v>1</v>
       </c>
       <c r="F26" s="7">
         <v>0</v>
       </c>
-      <c r="G26" s="18" t="s">
-        <v>193</v>
+      <c r="G26" s="7" t="b">
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="H26" s="7">
         <v>1</v>
       </c>
       <c r="I26" s="8" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="J26" s="8" t="s">
         <v>51</v>
@@ -4251,7 +4141,7 @@
         <v>54</v>
       </c>
       <c r="O26" s="9" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="P26" s="8" t="s">
         <v>56</v>
@@ -4293,7 +4183,7 @@
         <v>57</v>
       </c>
       <c r="AC26" s="7">
-        <v>0.092</v>
+        <v>9.1999999999999998E-2</v>
       </c>
       <c r="AD26" s="8" t="s">
         <v>57</v>
@@ -4317,7 +4207,7 @@
         <v>61</v>
       </c>
       <c r="AK26" s="8" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="AL26" s="8" t="s">
         <v>59</v>
@@ -4329,10 +4219,10 @@
         <v>63</v>
       </c>
       <c r="AO26" s="8" t="s">
-        <v>64</v>
+        <v>187</v>
       </c>
       <c r="AP26" s="8" t="s">
-        <v>64</v>
+        <v>189</v>
       </c>
       <c r="AQ26" s="8" t="s">
         <v>64</v>
@@ -4347,31 +4237,34 @@
         <v>68</v>
       </c>
     </row>
-    <row r="27" ht="18.75" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="7"/>
       <c r="B27" s="8" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="C27" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="D27" s="7">
+      <c r="D27" s="7" t="b">
         <f>TRUE()</f>
-      </c>
-      <c r="E27" s="7">
+        <v>1</v>
+      </c>
+      <c r="E27" s="7" t="b">
         <f>TRUE()</f>
+        <v>1</v>
       </c>
       <c r="F27" s="7">
         <v>0</v>
       </c>
-      <c r="G27" s="7">
+      <c r="G27" s="7" t="b">
         <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="H27" s="7">
         <v>1</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>194</v>
+        <v>50</v>
       </c>
       <c r="J27" s="8" t="s">
         <v>51</v>
@@ -4380,7 +4273,7 @@
         <v>52</v>
       </c>
       <c r="L27" s="7">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="M27" s="8" t="s">
         <v>53</v>
@@ -4389,7 +4282,7 @@
         <v>54</v>
       </c>
       <c r="O27" s="9" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="P27" s="8" t="s">
         <v>56</v>
@@ -4401,16 +4294,16 @@
         <v>58</v>
       </c>
       <c r="S27" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T27" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U27" s="10">
-        <v>0.65</v>
+        <v>0.4</v>
       </c>
       <c r="V27" s="7">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="W27" s="8" t="s">
         <v>57</v>
@@ -4431,7 +4324,7 @@
         <v>57</v>
       </c>
       <c r="AC27" s="7">
-        <v>0.092</v>
+        <v>9.1999999999999998E-2</v>
       </c>
       <c r="AD27" s="8" t="s">
         <v>57</v>
@@ -4455,7 +4348,7 @@
         <v>61</v>
       </c>
       <c r="AK27" s="8" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="AL27" s="8" t="s">
         <v>59</v>
@@ -4467,7 +4360,7 @@
         <v>63</v>
       </c>
       <c r="AO27" s="8" t="s">
-        <v>197</v>
+        <v>64</v>
       </c>
       <c r="AP27" s="8" t="s">
         <v>64</v>
@@ -4475,8 +4368,8 @@
       <c r="AQ27" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="AR27" s="11" t="s">
-        <v>66</v>
+      <c r="AR27" s="8" t="s">
+        <v>192</v>
       </c>
       <c r="AS27" s="8" t="s">
         <v>67</v>
@@ -4485,31 +4378,34 @@
         <v>68</v>
       </c>
     </row>
-    <row r="28" ht="18.75" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="7"/>
       <c r="B28" s="8" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="C28" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="D28" s="7">
+      <c r="D28" s="7" t="b">
         <f>TRUE()</f>
-      </c>
-      <c r="E28" s="7">
+        <v>1</v>
+      </c>
+      <c r="E28" s="7" t="b">
         <f>TRUE()</f>
+        <v>1</v>
       </c>
       <c r="F28" s="7">
         <v>0</v>
       </c>
-      <c r="G28" s="7">
+      <c r="G28" s="7" t="b">
         <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="H28" s="7">
         <v>1</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>194</v>
+        <v>50</v>
       </c>
       <c r="J28" s="8" t="s">
         <v>51</v>
@@ -4518,7 +4414,7 @@
         <v>52</v>
       </c>
       <c r="L28" s="7">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="M28" s="8" t="s">
         <v>53</v>
@@ -4527,7 +4423,7 @@
         <v>54</v>
       </c>
       <c r="O28" s="9" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="P28" s="8" t="s">
         <v>56</v>
@@ -4539,16 +4435,16 @@
         <v>58</v>
       </c>
       <c r="S28" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T28" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U28" s="10">
-        <v>0.65</v>
+        <v>0.4</v>
       </c>
       <c r="V28" s="7">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="W28" s="8" t="s">
         <v>57</v>
@@ -4569,7 +4465,7 @@
         <v>57</v>
       </c>
       <c r="AC28" s="7">
-        <v>0.092</v>
+        <v>9.1999999999999998E-2</v>
       </c>
       <c r="AD28" s="8" t="s">
         <v>57</v>
@@ -4593,7 +4489,7 @@
         <v>61</v>
       </c>
       <c r="AK28" s="8" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="AL28" s="8" t="s">
         <v>59</v>
@@ -4605,16 +4501,16 @@
         <v>63</v>
       </c>
       <c r="AO28" s="8" t="s">
-        <v>64</v>
+        <v>187</v>
       </c>
       <c r="AP28" s="8" t="s">
-        <v>199</v>
+        <v>64</v>
       </c>
       <c r="AQ28" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="AR28" s="11" t="s">
-        <v>66</v>
+      <c r="AR28" s="8" t="s">
+        <v>192</v>
       </c>
       <c r="AS28" s="8" t="s">
         <v>67</v>
@@ -4623,31 +4519,34 @@
         <v>68</v>
       </c>
     </row>
-    <row r="29" ht="18.75" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="7"/>
       <c r="B29" s="8" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="C29" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="D29" s="7">
+      <c r="D29" s="7" t="b">
         <f>TRUE()</f>
-      </c>
-      <c r="E29" s="7">
+        <v>1</v>
+      </c>
+      <c r="E29" s="7" t="b">
         <f>TRUE()</f>
+        <v>1</v>
       </c>
       <c r="F29" s="7">
         <v>0</v>
       </c>
-      <c r="G29" s="7">
+      <c r="G29" s="7" t="b">
         <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="H29" s="7">
         <v>1</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>194</v>
+        <v>50</v>
       </c>
       <c r="J29" s="8" t="s">
         <v>51</v>
@@ -4656,7 +4555,7 @@
         <v>52</v>
       </c>
       <c r="L29" s="7">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="M29" s="8" t="s">
         <v>53</v>
@@ -4665,7 +4564,7 @@
         <v>54</v>
       </c>
       <c r="O29" s="9" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="P29" s="8" t="s">
         <v>56</v>
@@ -4677,16 +4576,16 @@
         <v>58</v>
       </c>
       <c r="S29" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T29" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U29" s="10">
-        <v>0.65</v>
+        <v>0.4</v>
       </c>
       <c r="V29" s="7">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="W29" s="8" t="s">
         <v>57</v>
@@ -4707,7 +4606,7 @@
         <v>57</v>
       </c>
       <c r="AC29" s="7">
-        <v>0.092</v>
+        <v>9.1999999999999998E-2</v>
       </c>
       <c r="AD29" s="8" t="s">
         <v>57</v>
@@ -4731,7 +4630,7 @@
         <v>61</v>
       </c>
       <c r="AK29" s="8" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="AL29" s="8" t="s">
         <v>59</v>
@@ -4743,16 +4642,16 @@
         <v>63</v>
       </c>
       <c r="AO29" s="8" t="s">
-        <v>197</v>
+        <v>64</v>
       </c>
       <c r="AP29" s="8" t="s">
-        <v>199</v>
+        <v>65</v>
       </c>
       <c r="AQ29" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="AR29" s="11" t="s">
-        <v>66</v>
+      <c r="AR29" s="8" t="s">
+        <v>192</v>
       </c>
       <c r="AS29" s="8" t="s">
         <v>67</v>
@@ -4761,25 +4660,28 @@
         <v>68</v>
       </c>
     </row>
-    <row r="30" ht="18.75" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:46" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="7"/>
       <c r="B30" s="8" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="C30" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="D30" s="7">
+      <c r="D30" s="7" t="b">
         <f>TRUE()</f>
-      </c>
-      <c r="E30" s="7">
+        <v>1</v>
+      </c>
+      <c r="E30" s="7" t="b">
         <f>TRUE()</f>
+        <v>1</v>
       </c>
       <c r="F30" s="7">
         <v>0</v>
       </c>
-      <c r="G30" s="7">
+      <c r="G30" s="7" t="b">
         <f>FALSE()</f>
+        <v>0</v>
       </c>
       <c r="H30" s="7">
         <v>1</v>
@@ -4803,7 +4705,7 @@
         <v>54</v>
       </c>
       <c r="O30" s="9" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="P30" s="8" t="s">
         <v>56</v>
@@ -4845,7 +4747,7 @@
         <v>57</v>
       </c>
       <c r="AC30" s="7">
-        <v>0.092</v>
+        <v>9.1999999999999998E-2</v>
       </c>
       <c r="AD30" s="8" t="s">
         <v>57</v>
@@ -4869,7 +4771,7 @@
         <v>61</v>
       </c>
       <c r="AK30" s="8" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="AL30" s="8" t="s">
         <v>59</v>
@@ -4881,440 +4783,26 @@
         <v>63</v>
       </c>
       <c r="AO30" s="8" t="s">
-        <v>64</v>
+        <v>187</v>
       </c>
       <c r="AP30" s="8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AQ30" s="8" t="s">
         <v>64</v>
       </c>
       <c r="AR30" s="8" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="AS30" s="8" t="s">
         <v>67</v>
       </c>
       <c r="AT30" s="8" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="31" ht="18.75" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
-      <c r="A31" s="7"/>
-      <c r="B31" s="8" t="s">
-        <v>203</v>
-      </c>
-      <c r="C31" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="D31" s="7">
-        <f>TRUE()</f>
-      </c>
-      <c r="E31" s="7">
-        <f>TRUE()</f>
-      </c>
-      <c r="F31" s="7">
-        <v>0</v>
-      </c>
-      <c r="G31" s="7">
-        <f>FALSE()</f>
-      </c>
-      <c r="H31" s="7">
-        <v>1</v>
-      </c>
-      <c r="I31" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="J31" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="K31" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="L31" s="7">
-        <v>1</v>
-      </c>
-      <c r="M31" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="N31" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="O31" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="P31" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="Q31" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="R31" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="S31" s="7">
-        <v>0</v>
-      </c>
-      <c r="T31" s="7">
-        <v>0</v>
-      </c>
-      <c r="U31" s="10">
-        <v>0.4</v>
-      </c>
-      <c r="V31" s="7">
-        <v>1.5</v>
-      </c>
-      <c r="W31" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="X31" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="Y31" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="Z31" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AA31" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AB31" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="AC31" s="7">
-        <v>0.092</v>
-      </c>
-      <c r="AD31" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="AE31" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AF31" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AG31" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AH31" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AI31" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AJ31" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="AK31" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL31" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AM31" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AN31" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="AO31" s="8" t="s">
-        <v>197</v>
-      </c>
-      <c r="AP31" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="AQ31" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="AR31" s="8" t="s">
-        <v>202</v>
-      </c>
-      <c r="AS31" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="AT31" s="8" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="32" ht="18.75" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
-      <c r="A32" s="7"/>
-      <c r="B32" s="8" t="s">
-        <v>204</v>
-      </c>
-      <c r="C32" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="D32" s="7">
-        <f>TRUE()</f>
-      </c>
-      <c r="E32" s="7">
-        <f>TRUE()</f>
-      </c>
-      <c r="F32" s="7">
-        <v>0</v>
-      </c>
-      <c r="G32" s="7">
-        <f>FALSE()</f>
-      </c>
-      <c r="H32" s="7">
-        <v>1</v>
-      </c>
-      <c r="I32" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="J32" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="K32" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="L32" s="7">
-        <v>1</v>
-      </c>
-      <c r="M32" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="N32" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="O32" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="P32" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="Q32" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="R32" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="S32" s="7">
-        <v>0</v>
-      </c>
-      <c r="T32" s="7">
-        <v>0</v>
-      </c>
-      <c r="U32" s="10">
-        <v>0.4</v>
-      </c>
-      <c r="V32" s="7">
-        <v>1.5</v>
-      </c>
-      <c r="W32" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="X32" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="Y32" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="Z32" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AA32" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AB32" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="AC32" s="7">
-        <v>0.092</v>
-      </c>
-      <c r="AD32" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="AE32" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AF32" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AG32" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AH32" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AI32" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AJ32" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="AK32" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL32" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AM32" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AN32" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="AO32" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="AP32" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="AQ32" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="AR32" s="8" t="s">
-        <v>202</v>
-      </c>
-      <c r="AS32" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="AT32" s="8" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="33" ht="18.75" customHeight="1" spans="1:46" x14ac:dyDescent="0.25">
-      <c r="A33" s="7"/>
-      <c r="B33" s="8" t="s">
-        <v>205</v>
-      </c>
-      <c r="C33" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="D33" s="7">
-        <f>TRUE()</f>
-      </c>
-      <c r="E33" s="7">
-        <f>TRUE()</f>
-      </c>
-      <c r="F33" s="7">
-        <v>0</v>
-      </c>
-      <c r="G33" s="7">
-        <f>FALSE()</f>
-      </c>
-      <c r="H33" s="7">
-        <v>1</v>
-      </c>
-      <c r="I33" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="J33" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="K33" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="L33" s="7">
-        <v>1</v>
-      </c>
-      <c r="M33" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="N33" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="O33" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="P33" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="Q33" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="R33" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="S33" s="7">
-        <v>0</v>
-      </c>
-      <c r="T33" s="7">
-        <v>0</v>
-      </c>
-      <c r="U33" s="10">
-        <v>0.4</v>
-      </c>
-      <c r="V33" s="7">
-        <v>1.5</v>
-      </c>
-      <c r="W33" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="X33" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="Y33" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="Z33" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AA33" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AB33" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="AC33" s="7">
-        <v>0.092</v>
-      </c>
-      <c r="AD33" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="AE33" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AF33" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AG33" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AH33" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AI33" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AJ33" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="AK33" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL33" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AM33" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="AN33" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="AO33" s="8" t="s">
-        <v>197</v>
-      </c>
-      <c r="AP33" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="AQ33" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="AR33" s="8" t="s">
-        <v>202</v>
-      </c>
-      <c r="AS33" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="AT33" s="8" t="s">
         <v>68</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>